<commit_message>
updated already existing indicators and included labour
</commit_message>
<xml_diff>
--- a/MPI_10092026/Africa_MPI_Collector_Progress_Report.xlsx
+++ b/MPI_10092026/Africa_MPI_Collector_Progress_Report.xlsx
@@ -915,7 +915,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>static_url (Tier-1 API)</t>
+          <t>NSO data API, 3 table(s) (Tier-1 API)</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>NSO (NBS)</t>
+          <t>NSO (National Bureau of Statistics)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">

</xml_diff>